<commit_message>
NAKO-3 DPEs and DD of NAKO
</commit_message>
<xml_diff>
--- a/analyst/Tracy/rmonize/data_dictionary/DD_NAKO_TRACY.xlsx
+++ b/analyst/Tracy/rmonize/data_dictionary/DD_NAKO_TRACY.xlsx
@@ -1,22 +1,198 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Tracy\rmonize\data_dictionary\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E98004-0A4A-4DEF-8EF7-AD8640C0DD1F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
     <sheet name="Categories" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="55">
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>label</t>
+  </si>
+  <si>
+    <t>valueType</t>
+  </si>
+  <si>
+    <t>variable</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID </t>
+  </si>
+  <si>
+    <t>integer</t>
+  </si>
+  <si>
+    <t>basis_sex</t>
+  </si>
+  <si>
+    <t>Geschlecht</t>
+  </si>
+  <si>
+    <t>Alter am Erhebungsdatum</t>
+  </si>
+  <si>
+    <t>decimal</t>
+  </si>
+  <si>
+    <t>basis_age</t>
+  </si>
+  <si>
+    <t>a_ses_isced11_level</t>
+  </si>
+  <si>
+    <t>Bildungsniveau nach ISCED 2011</t>
+  </si>
+  <si>
+    <t>Less than primary education (Not applicable for Germany)</t>
+  </si>
+  <si>
+    <t>Primary education</t>
+  </si>
+  <si>
+    <t>Lower secondary education</t>
+  </si>
+  <si>
+    <t>Upper secondary education</t>
+  </si>
+  <si>
+    <t>Post-secondary non-tertiary education</t>
+  </si>
+  <si>
+    <t>Short-cycle tertiary education (Not applicable for Germany)</t>
+  </si>
+  <si>
+    <t>Bachelor's or equivalent level</t>
+  </si>
+  <si>
+    <t>Master's or equivalent level</t>
+  </si>
+  <si>
+    <t>Doctoral or equivalent level</t>
+  </si>
+  <si>
+    <t>Weiblich</t>
+  </si>
+  <si>
+    <t>Mannlich</t>
+  </si>
+  <si>
+    <t>a_gpaq_ptotalmet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rauchstatus </t>
+  </si>
+  <si>
+    <t>Kein Raucher, auch nicht ehemalig</t>
+  </si>
+  <si>
+    <t>Ehemaliger Raucher</t>
+  </si>
+  <si>
+    <t>Raucher</t>
+  </si>
+  <si>
+    <t>Rauchstatus unbekannt</t>
+  </si>
+  <si>
+    <t>a_smok_stat_qn</t>
+  </si>
+  <si>
+    <t>d_sn1</t>
+  </si>
+  <si>
+    <t>Wie viele Kinder haben Sie</t>
+  </si>
+  <si>
+    <t>a_f_smok_quit_age</t>
+  </si>
+  <si>
+    <t>Alter Rauchende</t>
+  </si>
+  <si>
+    <t>d_an_ca</t>
+  </si>
+  <si>
+    <t>Wurde bei Ihnen jemals von einem Arzt eine Krebserkrankung diagnostiziert?</t>
+  </si>
+  <si>
+    <t>Ja</t>
+  </si>
+  <si>
+    <t>Nein</t>
+  </si>
+  <si>
+    <t>d_an_cv_6</t>
+  </si>
+  <si>
+    <t>Bluthochdruck</t>
+  </si>
+  <si>
+    <t>d_f_mp1</t>
+  </si>
+  <si>
+    <t>d_fa_m3_dm</t>
+  </si>
+  <si>
+    <t>Diabetes mellitus (Zuckerkrankheit)</t>
+  </si>
+  <si>
+    <t>Ja, aber Alter unbekannt</t>
+  </si>
+  <si>
+    <t>Ja, jÃ¼nger als 40 Jahre</t>
+  </si>
+  <si>
+    <t>Ja, zwischen 40 und 59 Jahren</t>
+  </si>
+  <si>
+    <t>d_an_cv_6_fu</t>
+  </si>
+  <si>
+    <t>MET-Min./Woche kärperl. Aktivität gesamt</t>
+  </si>
+  <si>
+    <t>a_packyears</t>
+  </si>
+  <si>
+    <t>Smoking intensity as number of packyears</t>
+  </si>
+  <si>
+    <t>Haben Sie jemals Hormonersatzpräparate aufgrund Ihrer Wechseljahre oder aufgrund des Ausbleibens Ihrer Regelblutung eingenommen</t>
+  </si>
+  <si>
+    <t>Ja, 60 Jahre und Ãlter</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,6 +204,19 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -53,17 +242,45 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -110,7 +327,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -142,9 +359,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -176,6 +411,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -351,57 +604,492 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="19.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>index</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>valueType</t>
-        </is>
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>44</v>
+      </c>
+      <c r="C14" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="57.5703125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>variable</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>label</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11">
+        <v>7</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12">
+        <v>8</v>
+      </c>
+      <c r="C12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13">
+        <v>1</v>
+      </c>
+      <c r="C13" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17">
+        <v>2</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19">
+        <v>12</v>
+      </c>
+      <c r="C19" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B20">
+        <v>13</v>
+      </c>
+      <c r="C20" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21">
+        <v>14</v>
+      </c>
+      <c r="C21" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25">
+        <v>2</v>
+      </c>
+      <c r="C25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27">
+        <v>2</v>
+      </c>
+      <c r="C27" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>